<commit_message>
Catalogo completo: 197 productos con variantes reflejadas (tallas, colores y estampados como chips) y galerias de hasta 4 fotos donde aplican; joyas 3 por coleccion, toda la moda valida, juguetes 24, escolar completa, bebe 30 y todos los combos; hero y favoritos actualizados
</commit_message>
<xml_diff>
--- a/Gava_Joyeria_Catalogo.xlsx
+++ b/Gava_Joyeria_Catalogo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Catálogo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catálogo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$P$898</definedName>
@@ -54256,7 +54256,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-13 06:25</t>
+          <t>2026-10-13 02:14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Open Mind como 5o proveedor (tiendasopenmind.com): 23 prendas urbanas (camisetas, camibusos, bermudas) en categoria Ropa urbana + favoritos; campo prov en los 1824 productos y toggles por catalogo de proveedor en el admin (oculta gava/majestic/taiwan/solobabys/openmind); Excel OpenMind_Catalogo.xlsx generado por el sync
</commit_message>
<xml_diff>
--- a/Gava_Joyeria_Catalogo.xlsx
+++ b/Gava_Joyeria_Catalogo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Catálogo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catálogo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$P$898</definedName>
@@ -54256,7 +54256,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-13 12:24</t>
+          <t>2026-10-13 08:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Marca unica ante el cliente: cero menciones de proveedores (lineas internas l1-l5 en catalogo y admin, comentarios neutrales) y 1247 imagenes rehospedadas a img/p/ (ningun dominio ajeno en las fotos); footer Tienda con las 7 categorias en orden de conversion; favoritos protagonistas con 2 filas y tarjetas mas grandes; FAB de compartir visible en movil; admin con 6 toggles de carrusel nombrados dinamicamente con su categoria y conteo actuales
</commit_message>
<xml_diff>
--- a/Gava_Joyeria_Catalogo.xlsx
+++ b/Gava_Joyeria_Catalogo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Catálogo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catálogo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$P$894</definedName>
@@ -54024,7 +54024,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-13 18:24</t>
+          <t>2026-10-13 14:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pendientes de syncs previos: README con la fila de la suite qa_aterrizaje_precios.js y los 5 Excel regenerados en la corrida del rehost de imagenes de Majestic
</commit_message>
<xml_diff>
--- a/Gava_Joyeria_Catalogo.xlsx
+++ b/Gava_Joyeria_Catalogo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Catálogo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catálogo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo'!$A$1:$P$919</definedName>
@@ -55670,7 +55670,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-21 12:35</t>
+          <t>2026-10-21 08:02</t>
         </is>
       </c>
     </row>

</xml_diff>